<commit_message>
🗑️ Deprecate Parameter option non_negative
</commit_message>
<xml_diff>
--- a/glotaran/builtin/io/pandas/test/data/reference_parameters_alternative_notation.xlsx
+++ b/glotaran/builtin/io/pandas/test/data/reference_parameters_alternative_notation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
   <si>
     <t xml:space="preserve">Label</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t xml:space="preserve">Min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non-negative</t>
   </si>
   <si>
     <t xml:space="preserve">Vary</t>
@@ -195,14 +192,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -227,132 +224,109 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="3" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="3" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G4" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H4" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G6" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="3" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>1</v>
@@ -361,32 +335,24 @@
         <v>-1</v>
       </c>
       <c r="G7" s="3" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>11</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G8" s="3" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>

</xml_diff>